<commit_message>
- data converter : buildable & runnable
</commit_message>
<xml_diff>
--- a/StaticData/XLSX/Item/item.xlsx
+++ b/StaticData/XLSX/Item/item.xlsx
@@ -6,7 +6,7 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Item" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -16,12 +16,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>qwer</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>ID(int)</t>
+  </si>
+  <si>
+    <t>Name(string)</t>
+  </si>
+  <si>
+    <t>Effect(string)</t>
+  </si>
+  <si>
+    <t>Cost(int)</t>
+  </si>
+  <si>
+    <t>RedPotion</t>
+  </si>
+  <si>
+    <t>HealHP</t>
+  </si>
+  <si>
+    <t>BluePotion</t>
+  </si>
+  <si>
+    <t>HealMP</t>
   </si>
 </sst>
 </file>
@@ -36,12 +54,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor theme="9" tint="0.59999389629810485"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,8 +80,14 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,27 +586,53 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" min="1" max="1" width="6.00390625"/>
+    <col bestFit="1" min="2" max="2" width="11.7109375"/>
+    <col bestFit="1" min="3" max="3" width="11.421875"/>
+    <col bestFit="1" min="4" max="4" width="8.00390625"/>
+  </cols>
   <sheetData>
-    <row r="1" ht="14.25">
-      <c r="A1">
-        <v>11</v>
-      </c>
-      <c r="B1">
-        <v>22</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" s="1" customFormat="1" ht="14.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D1">
-        <v>5.2999999999999998</v>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" ht="14.25">
-      <c r="A2" t="s">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>112</v>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="4">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>